<commit_message>
feat: complete SSIEMS CSE Academic Portal with unified UI/UX, year-wise directory, and faculty leave management
</commit_message>
<xml_diff>
--- a/backend/Result_Sheet.xlsx
+++ b/backend/Result_Sheet.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marksheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Marksheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,12 +434,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -449,14 +449,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Elective – VIII (DL) - Mid Semester - Marksheet</t>
+          <t>Data Structures - Mid Semester - Marksheet</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Subject: Elective – VIII (DL)</t>
+          <t>Subject: Data Structures</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Class: BE (BTech-CSE)</t>
+          <t>Class: SY-CSE</t>
         </is>
       </c>
     </row>
@@ -528,332 +528,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PRN-2122521242046</t>
+          <t>CS225201</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SYED RAYYAN SYED FARHANUDDIN</t>
+          <t>AMBHORE VAISHNAVI LIMBAJI</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>prn-2122521242046@college.edu</t>
+          <t>cs225201@college.edu</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
         <v>20</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
-        <is>
-          <t>Checked</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>PRN-2222521242013</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>BHAKRE VAISHNAVI SHESHARAO</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>prn-2222521242013@college.edu</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>9</v>
-      </c>
-      <c r="E10" t="n">
-        <v>20</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>45.0%</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Checked</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>PRN-2222521242060</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>INGOLE KARAN SADASHIV</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>prn-2222521242060@college.edu</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>20</v>
-      </c>
-      <c r="E11" t="n">
-        <v>20</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Checked</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>PRN-2222521242012</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>JADHAV RITIKA VIAJAY</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>prn-2222521242012@college.edu</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Not Graded</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>20</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>PRN-2222521242009</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>RATHOD KALPANA BALAJI</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>prn-2222521242009@college.edu</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>14</v>
-      </c>
-      <c r="E13" t="n">
-        <v>20</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>70.0%</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Checked</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>PRN-2222521242020</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>BULBULE SWATI RAMESHRAO</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>prn-2222521242020@college.edu</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Not Graded</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>20</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>PRN-2122521242035</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>SHAIKH TAHZEEB SHAIKH NAYEEM</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>prn-2122521242035@college.edu</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>14</v>
-      </c>
-      <c r="E15" t="n">
-        <v>20</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>70.0%</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Checked</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>PRN-2222521242026</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>WAVDHANE PRANITA BHAGWAN</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>prn-2222521242026@college.edu</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>6</v>
-      </c>
-      <c r="E16" t="n">
-        <v>20</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>30.0%</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Checked</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>PRN-2022521242021</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>SANIYA KAUSER MAROOF SHAIKH</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>prn-2022521242021@college.edu</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>17</v>
-      </c>
-      <c r="E17" t="n">
-        <v>20</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>85.0%</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Checked</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>PRN-2222521242001</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>ZADE VISHAL SUNIL</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>prn-2222521242001@college.edu</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>13</v>
-      </c>
-      <c r="E18" t="n">
-        <v>20</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>65.0%</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
         <is>
           <t>Checked</t>
         </is>

</xml_diff>